<commit_message>
modify post validation and mail send part
</commit_message>
<xml_diff>
--- a/output/AMER_Intercompny/Output/AMER_Intercompany billing lines_April 2026.xlsx
+++ b/output/AMER_Intercompny/Output/AMER_Intercompany billing lines_April 2026.xlsx
@@ -1949,7 +1949,7 @@
       <c r="E10" s="177" t="n"/>
       <c r="F10" s="178" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="G10" s="179" t="n"/>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Offering of Crowne Plaza Power Up Mornings Breakfast Program Workshop (Spanish)</t>
+          <t>Offering of Crowne Plaza 'Power Up Mornings' Breakfast Program Workshop (Spanish)</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I33" t="n">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -10510,7 +10510,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Offering of Crowne Plaza Power Up Mornings Breakfast Program Workshop (Spanish)</t>
+          <t>Offering of Crowne Plaza 'Power Up Mornings' Breakfast Program Workshop (Spanish)</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -12687,7 +12687,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I91" t="n">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -14013,7 +14013,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I105" t="n">
@@ -19600,7 +19600,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I164" t="n">
@@ -21209,7 +21209,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I181" t="n">
@@ -23762,7 +23762,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I208" t="n">
@@ -24142,7 +24142,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I212" t="n">
@@ -24617,7 +24617,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I217" t="n">
@@ -24900,7 +24900,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I220" t="n">
@@ -25088,7 +25088,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I222" t="n">
@@ -26980,7 +26980,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I242" t="n">
@@ -30677,7 +30677,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I281" t="n">
@@ -33806,7 +33806,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I314" t="n">
@@ -34091,7 +34091,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I317" t="n">
@@ -34281,7 +34281,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I319" t="n">
@@ -35419,7 +35419,7 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I331" t="n">
@@ -36082,7 +36082,7 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I338" t="n">
@@ -39300,7 +39300,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I372" t="n">
@@ -42425,7 +42425,7 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I405" t="n">
@@ -44511,7 +44511,7 @@
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I427" t="n">
@@ -44792,7 +44792,7 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I430" t="n">
@@ -47632,7 +47632,7 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I460" t="n">
@@ -54644,7 +54644,7 @@
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I534" t="n">
@@ -55022,7 +55022,7 @@
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I538" t="n">
@@ -55212,7 +55212,7 @@
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I540" t="n">
@@ -55495,7 +55495,7 @@
       </c>
       <c r="H543" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I543" t="n">
@@ -55685,7 +55685,7 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I545" t="n">
@@ -56730,7 +56730,7 @@
       </c>
       <c r="H556" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I556" t="n">
@@ -57674,7 +57674,7 @@
       </c>
       <c r="H566" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I566" t="n">
@@ -61842,7 +61842,7 @@
       </c>
       <c r="H610" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC (Spanish)</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC (Spanish)</t>
         </is>
       </c>
       <c r="I610" t="n">
@@ -62127,7 +62127,7 @@
       </c>
       <c r="H613" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I613" t="n">
@@ -62222,7 +62222,7 @@
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>Offering of Revenue Management Essentials Certification Part Two  RMEC</t>
+          <t>Offering of Revenue Management Essentials Certification Part Two â€“ RMEC</t>
         </is>
       </c>
       <c r="I614" t="n">

</xml_diff>